<commit_message>
adapted mortality rate and excretion rate of fauna
</commit_message>
<xml_diff>
--- a/parameters.xlsx
+++ b/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\freefilesyncHBU\projects\git\gw_ecosystem_services\Fulda_plains\R_git\gtm_River_Fulda_floodplain\gtm_River_Fulda_floodplain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920A823B-A0F9-467B-ABDD-6094D82855CB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23170355-5709-4846-A6D2-985693089006}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="504" windowWidth="23040" windowHeight="7140" xr2:uid="{8E85E7A9-C450-5844-BD64-77EB6910F2CD}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="calculating_COD" sheetId="6" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$A$3:$AJ$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$A$3:$AI$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -88,7 +88,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD3" authorId="0" shapeId="0" xr:uid="{C3505123-F90F-DE41-BEE8-86A5DB659096}">
+    <comment ref="AC3" authorId="0" shapeId="0" xr:uid="{C3505123-F90F-DE41-BEE8-86A5DB659096}">
       <text>
         <r>
           <rPr>
@@ -247,7 +247,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z4" authorId="3" shapeId="0" xr:uid="{B2EEDDFE-EFB6-B841-B3B1-49218DCB8340}">
+    <comment ref="Y4" authorId="3" shapeId="0" xr:uid="{B2EEDDFE-EFB6-B841-B3B1-49218DCB8340}">
       <text>
         <r>
           <rPr>
@@ -310,7 +310,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE4" authorId="4" shapeId="0" xr:uid="{D83D8722-287D-8543-91DC-DFD968583D4B}">
+    <comment ref="AD4" authorId="4" shapeId="0" xr:uid="{D83D8722-287D-8543-91DC-DFD968583D4B}">
       <text>
         <r>
           <rPr>
@@ -323,7 +323,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -407,7 +407,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z5" authorId="7" shapeId="0" xr:uid="{944B0A6E-7F35-8040-8354-541096ED2DBE}">
+    <comment ref="Y5" authorId="7" shapeId="0" xr:uid="{944B0A6E-7F35-8040-8354-541096ED2DBE}">
       <text>
         <r>
           <rPr>
@@ -424,7 +424,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE5" authorId="4" shapeId="0" xr:uid="{853BCBCA-AD94-4092-B9D5-CDE911D53FC2}">
+    <comment ref="AD5" authorId="4" shapeId="0" xr:uid="{16668028-E470-49D8-A575-5BF14B51E0D7}">
       <text>
         <r>
           <rPr>
@@ -437,7 +437,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -521,7 +521,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z6" authorId="10" shapeId="0" xr:uid="{4659E4E8-C0C9-CB4D-BEA9-CCB12CD16D5B}">
+    <comment ref="Y6" authorId="10" shapeId="0" xr:uid="{4659E4E8-C0C9-CB4D-BEA9-CCB12CD16D5B}">
       <text>
         <r>
           <rPr>
@@ -538,7 +538,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE6" authorId="4" shapeId="0" xr:uid="{51AED2A8-D3B7-403D-AA5A-200DCAABACFA}">
+    <comment ref="AD6" authorId="4" shapeId="0" xr:uid="{2C3E63E2-3AE0-4A5B-8C7D-9BF28330D619}">
       <text>
         <r>
           <rPr>
@@ -551,7 +551,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -589,7 +589,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z7" authorId="13" shapeId="0" xr:uid="{D9858DC7-D04C-4A4F-872C-0C59D675639A}">
+    <comment ref="Y7" authorId="13" shapeId="0" xr:uid="{D9858DC7-D04C-4A4F-872C-0C59D675639A}">
       <text>
         <r>
           <rPr>
@@ -606,7 +606,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE7" authorId="4" shapeId="0" xr:uid="{336D7F98-AD70-4487-9E19-A2872968D1C6}">
+    <comment ref="AD7" authorId="4" shapeId="0" xr:uid="{52E6596C-BF01-40FE-80EF-E81EF72B1B0A}">
       <text>
         <r>
           <rPr>
@@ -619,7 +619,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -703,7 +703,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z8" authorId="16" shapeId="0" xr:uid="{8ABD701E-78D0-4A47-8F33-59280C42BAAB}">
+    <comment ref="Y8" authorId="16" shapeId="0" xr:uid="{8ABD701E-78D0-4A47-8F33-59280C42BAAB}">
       <text>
         <r>
           <rPr>
@@ -720,7 +720,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE8" authorId="4" shapeId="0" xr:uid="{2A45CBFD-6121-4554-8977-78E204540AE9}">
+    <comment ref="AD8" authorId="4" shapeId="0" xr:uid="{92E5DB6E-68AE-4BE9-AC60-965E4EFEF9C9}">
       <text>
         <r>
           <rPr>
@@ -733,7 +733,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -817,7 +817,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z9" authorId="19" shapeId="0" xr:uid="{74D124C3-18A4-4549-83DD-7E733D9BD57D}">
+    <comment ref="Y9" authorId="19" shapeId="0" xr:uid="{74D124C3-18A4-4549-83DD-7E733D9BD57D}">
       <text>
         <r>
           <rPr>
@@ -834,7 +834,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE9" authorId="4" shapeId="0" xr:uid="{AA8D6C3D-3E14-4946-A46D-8747516AE283}">
+    <comment ref="AD9" authorId="4" shapeId="0" xr:uid="{5B2AB557-5C4D-4A18-B601-D1F593004EA2}">
       <text>
         <r>
           <rPr>
@@ -847,7 +847,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -931,7 +931,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z10" authorId="19" shapeId="0" xr:uid="{5E9B9DF4-3124-4011-8650-F6C413EFC23B}">
+    <comment ref="Y10" authorId="19" shapeId="0" xr:uid="{5E9B9DF4-3124-4011-8650-F6C413EFC23B}">
       <text>
         <r>
           <rPr>
@@ -948,7 +948,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE10" authorId="4" shapeId="0" xr:uid="{86F3F138-07CF-4120-B34C-9F8AF0FDCE5B}">
+    <comment ref="AD10" authorId="4" shapeId="0" xr:uid="{3A5D2B68-C202-47CB-8961-7FC8DDCB5D87}">
       <text>
         <r>
           <rPr>
@@ -961,7 +961,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -1045,7 +1045,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z11" authorId="19" shapeId="0" xr:uid="{DD778B4E-FBBE-482A-A38D-F6A2FD45AD3D}">
+    <comment ref="Y11" authorId="19" shapeId="0" xr:uid="{DD778B4E-FBBE-482A-A38D-F6A2FD45AD3D}">
       <text>
         <r>
           <rPr>
@@ -1062,7 +1062,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE11" authorId="4" shapeId="0" xr:uid="{24967105-65BC-4B43-B982-22847566800B}">
+    <comment ref="AD11" authorId="4" shapeId="0" xr:uid="{48DA997C-8DFD-4B73-9E86-327CAC4DFDC5}">
       <text>
         <r>
           <rPr>
@@ -1075,7 +1075,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -1159,7 +1159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z12" authorId="19" shapeId="0" xr:uid="{5F6BAB42-F9A7-4880-A8DF-F9E5F4DEAA58}">
+    <comment ref="Y12" authorId="19" shapeId="0" xr:uid="{5F6BAB42-F9A7-4880-A8DF-F9E5F4DEAA58}">
       <text>
         <r>
           <rPr>
@@ -1176,7 +1176,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE12" authorId="4" shapeId="0" xr:uid="{DE302AD6-DC40-4C0E-98E6-EC607558285A}">
+    <comment ref="AD12" authorId="4" shapeId="0" xr:uid="{155DF592-3843-4EA8-9AB8-E5135E1BAF92}">
       <text>
         <r>
           <rPr>
@@ -1189,7 +1189,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -1273,7 +1273,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z13" authorId="19" shapeId="0" xr:uid="{131DF270-3C73-49B5-BD68-1F49168AEBBC}">
+    <comment ref="Y13" authorId="19" shapeId="0" xr:uid="{131DF270-3C73-49B5-BD68-1F49168AEBBC}">
       <text>
         <r>
           <rPr>
@@ -1290,7 +1290,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE13" authorId="4" shapeId="0" xr:uid="{6E879F82-2B4B-45FB-AB54-CD13EDAE8F66}">
+    <comment ref="AD13" authorId="4" shapeId="0" xr:uid="{B66749DF-A4F3-46FC-B53B-BE6D26C8C927}">
       <text>
         <r>
           <rPr>
@@ -1303,7 +1303,7 @@
           <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Equating organic carbon to biofilm, we used the growth rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day. Assuming that the maximum growth rate is 10 times as high, we set the the maximum growth rate of fauna on microorganisms to 0.02 / day.</t>
+    Equating organic carbon to biofilm, and bacterial uptake to growth, we used the uptake rate measured by (Foulquier et al., 2010) of 0.35 µg C bacteria / day and using a biomass molar mass of 24.6 g/mol (see above), 1.05 mol COD/mol biomass (see above) this translates to 1.4939E-08 mol COD bacteria / day. Multiplying with an average COD bacterial dry mass of 1.0e-05 mol COD / L, yields 0.002 / day.</t>
         </r>
       </text>
     </comment>
@@ -1312,7 +1312,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="188">
   <si>
     <t>variable_parameter</t>
   </si>
@@ -1375,9 +1375,6 @@
   </si>
   <si>
     <t>K_MO_at_temp</t>
-  </si>
-  <si>
-    <t>rMO_COD_uptake_h_at_lab_temperature</t>
   </si>
   <si>
     <t>rMO_COD_uptake_per_day_at_lab_temperature</t>
@@ -2371,9 +2368,6 @@
     <t xml:space="preserve">fraction of detritus  becoming  BOC </t>
   </si>
   <si>
-    <t>2 mol COD / mol acetate. 64 g COD / 60 g acetate, i.e. 1.067 g COD / g acetate</t>
-  </si>
-  <si>
     <t>microbial loss factor in scenarios where there is no fauna - i.e. cell respiration, grazing through the microbial loop, cell death etc.</t>
   </si>
   <si>
@@ -2386,9 +2380,6 @@
     <t>the factor how many times of TOC there is carbon bound in detritus; assuming that through soil passage, the TOC from precipitation is degraded, but a lot more detritus is mobilised</t>
   </si>
   <si>
-    <t>rate constant for bacterial uptake and oxidation of acetate Gerritse et al. (1992), assuming COD can be degraded like acetate, which is an error-prone assumption</t>
-  </si>
-  <si>
     <t>excretion rate of fauna; constant rate; excretion is biodegradable organic carbon (BOC) and added to that pool</t>
   </si>
   <si>
@@ -2405,6 +2396,9 @@
   </si>
   <si>
     <t>100% survival at 12 degrees, between 50 and 100% at 16 degrees, between 0 and50% at 20 degrees (Brielmann 2011). Assuming that half of the fauna population behaves like amphipods and half like asellids, 100% survival at 12 degrees, (75% survival at 16 degrees,) 25 % at 20 degrees. Taking the endpoint 20 degrees, 0.25 of the population survives after an increase by 8 degrees. This means that 0.75 have died. Thus , for each degree of increase, 0.75/8 = 0.09375 , roughly 1 % of the individuals die.    above or below 12 degree</t>
+  </si>
+  <si>
+    <t>rate constant per hour for bacterial uptake and oxidation of acetate Gerritse et al. (1992), assuming COD can be degraded like acetate, which is an error-prone assumption</t>
   </si>
 </sst>
 </file>
@@ -3073,7 +3067,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7B919E-F4BE-8A4F-9679-A3F32BFB830E}">
-  <dimension ref="A1:AJ13"/>
+  <dimension ref="A1:AI13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.69921875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="12.19921875" bestFit="1" customWidth="1"/>
@@ -3081,36 +3075,36 @@
     <col min="11" max="11" width="11.19921875" customWidth="1"/>
     <col min="13" max="13" width="11.19921875" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="12.19921875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="12.19921875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36">
+    <row r="1" spans="1:35">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G1" t="s">
+        <v>184</v>
+      </c>
+      <c r="H1" t="s">
+        <v>179</v>
+      </c>
+      <c r="L1" t="s">
         <v>180</v>
       </c>
-      <c r="G1" t="s">
-        <v>187</v>
-      </c>
-      <c r="H1" t="s">
-        <v>181</v>
-      </c>
-      <c r="L1" t="s">
-        <v>182</v>
-      </c>
       <c r="M1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="O1" t="s">
         <v>5</v>
@@ -3119,45 +3113,42 @@
         <v>17</v>
       </c>
       <c r="T1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="W1" t="s">
+        <v>187</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>87</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>182</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>177</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>185</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG1" t="s">
         <v>183</v>
       </c>
-      <c r="X1" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>185</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>179</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>188</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>184</v>
-      </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>186</v>
       </c>
-      <c r="AJ1" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="2" spans="1:36">
+    </row>
+    <row r="2" spans="1:35">
       <c r="C2" t="s">
         <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="N2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O2" t="s">
         <v>8</v>
@@ -3165,14 +3156,14 @@
       <c r="S2" t="s">
         <v>18</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AB2" t="s">
         <v>10</v>
       </c>
-      <c r="AF2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:36">
+      <c r="AE2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -3183,37 +3174,37 @@
         <v>4</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" t="s">
+        <v>75</v>
+      </c>
+      <c r="J3" t="s">
+        <v>42</v>
+      </c>
+      <c r="K3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L3" t="s">
         <v>28</v>
       </c>
-      <c r="I3" t="s">
-        <v>76</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="M3" t="s">
         <v>43</v>
       </c>
-      <c r="K3" t="s">
-        <v>75</v>
-      </c>
-      <c r="L3" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" t="s">
-        <v>44</v>
-      </c>
       <c r="N3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O3" t="s">
         <v>6</v>
@@ -3225,7 +3216,7 @@
         <v>9</v>
       </c>
       <c r="R3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S3" t="s">
         <v>16</v>
@@ -3240,49 +3231,46 @@
         <v>20</v>
       </c>
       <c r="W3" t="s">
-        <v>45</v>
-      </c>
-      <c r="X3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="X3" t="s">
         <v>21</v>
       </c>
       <c r="Y3" t="s">
+        <v>30</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AD3" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AA3" t="s">
+      <c r="AE3" t="s">
+        <v>25</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>13</v>
+      </c>
+      <c r="AG3" t="s">
         <v>50</v>
       </c>
-      <c r="AB3" t="s">
-        <v>55</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>23</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>13</v>
-      </c>
       <c r="AH3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AI3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:36">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:35">
       <c r="B4" s="4">
         <v>1</v>
       </c>
@@ -3335,7 +3323,7 @@
         <v>0</v>
       </c>
       <c r="R4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S4">
         <v>30</v>
@@ -3355,50 +3343,47 @@
       <c r="W4">
         <v>0.43</v>
       </c>
-      <c r="X4" s="4">
-        <f>W4*1.066</f>
-        <v>0.45838000000000001</v>
+      <c r="X4">
+        <f>W4 *24</f>
+        <v>10.32</v>
       </c>
       <c r="Y4">
-        <f>X4 *24</f>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z4">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA4">
+        <v>1E-4</v>
+      </c>
+      <c r="AB4">
         <v>1</v>
       </c>
-      <c r="AB4">
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>2E-3</v>
+      </c>
+      <c r="AE4">
+        <f>0.0001</f>
         <v>1E-4</v>
       </c>
-      <c r="AC4">
+      <c r="AF4">
+        <f>0.0001</f>
+        <v>1E-4</v>
+      </c>
+      <c r="AG4">
         <v>1</v>
       </c>
-      <c r="AD4">
-        <v>0</v>
-      </c>
-      <c r="AE4">
-        <v>2E-3</v>
-      </c>
-      <c r="AF4">
-        <v>1E-3</v>
-      </c>
-      <c r="AG4">
-        <f>0.001</f>
-        <v>1E-3</v>
-      </c>
-      <c r="AH4">
-        <v>1</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ4">
+      <c r="AH4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI4">
         <v>9.375E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:36">
+    <row r="5" spans="1:35">
       <c r="B5">
         <v>2</v>
       </c>
@@ -3451,7 +3436,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S5">
         <v>30</v>
@@ -3471,50 +3456,47 @@
       <c r="W5">
         <v>0.43</v>
       </c>
-      <c r="X5" s="4">
-        <f>W5*1.066</f>
-        <v>0.45838000000000001</v>
+      <c r="X5">
+        <f t="shared" ref="X5:X13" si="6">W5 *24</f>
+        <v>10.32</v>
       </c>
       <c r="Y5">
-        <f>X5 *24</f>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z5">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA5">
+        <v>1E-4</v>
+      </c>
+      <c r="AB5" s="21">
+        <v>0</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5">
+        <v>2E-3</v>
+      </c>
+      <c r="AE5">
+        <f t="shared" ref="AE5:AF13" si="7">0.0001</f>
+        <v>1E-4</v>
+      </c>
+      <c r="AF5">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AG5">
         <v>1</v>
       </c>
-      <c r="AB5">
-        <v>1E-4</v>
-      </c>
-      <c r="AC5" s="21">
-        <v>0</v>
-      </c>
-      <c r="AD5">
-        <v>0</v>
-      </c>
-      <c r="AE5">
-        <v>2E-3</v>
-      </c>
-      <c r="AF5">
-        <v>1E-3</v>
-      </c>
-      <c r="AG5">
-        <f t="shared" ref="AG5:AG13" si="6">0.001</f>
-        <v>1E-3</v>
-      </c>
-      <c r="AH5">
-        <v>1</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ5">
+      <c r="AH5" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI5">
         <v>9.375E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:36">
+    <row r="6" spans="1:35">
       <c r="B6">
         <v>3</v>
       </c>
@@ -3544,14 +3526,14 @@
         <v>1.0752025361042621</v>
       </c>
       <c r="K6">
-        <f t="shared" ref="K6:K9" si="7">J6/1000</f>
+        <f t="shared" ref="K6:K9" si="8">J6/1000</f>
         <v>1.075202536104262E-3</v>
       </c>
       <c r="L6" s="4">
         <v>10</v>
       </c>
       <c r="M6">
-        <f t="shared" ref="M6" si="8">L6*J6</f>
+        <f t="shared" ref="M6" si="9">L6*J6</f>
         <v>10.752025361042621</v>
       </c>
       <c r="N6">
@@ -3567,7 +3549,7 @@
         <v>0</v>
       </c>
       <c r="R6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S6">
         <v>30</v>
@@ -3577,7 +3559,7 @@
         <v>0.47258333333333336</v>
       </c>
       <c r="U6">
-        <f t="shared" ref="U6:U9" si="9">4.3 /1000000 *1.07</f>
+        <f t="shared" ref="U6:U9" si="10">4.3 /1000000 *1.07</f>
         <v>4.6009999999999997E-6</v>
       </c>
       <c r="V6">
@@ -3587,50 +3569,47 @@
       <c r="W6">
         <v>0.43</v>
       </c>
-      <c r="X6" s="4">
-        <f t="shared" ref="X6:X8" si="10">W6*1.066</f>
-        <v>0.45838000000000001</v>
+      <c r="X6">
+        <f t="shared" si="6"/>
+        <v>10.32</v>
       </c>
       <c r="Y6">
-        <f t="shared" ref="Y6:Y8" si="11">X6 *24</f>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z6">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA6">
+        <v>1E-4</v>
+      </c>
+      <c r="AB6">
         <v>1</v>
       </c>
-      <c r="AB6">
+      <c r="AC6">
+        <v>0</v>
+      </c>
+      <c r="AD6">
+        <v>2E-3</v>
+      </c>
+      <c r="AE6">
+        <f t="shared" si="7"/>
         <v>1E-4</v>
       </c>
-      <c r="AC6">
+      <c r="AF6">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AG6">
         <v>1</v>
       </c>
-      <c r="AD6">
-        <v>0</v>
-      </c>
-      <c r="AE6">
-        <v>2E-3</v>
-      </c>
-      <c r="AF6">
-        <v>1E-3</v>
-      </c>
-      <c r="AG6">
-        <f t="shared" si="6"/>
-        <v>1E-3</v>
-      </c>
-      <c r="AH6">
-        <v>1</v>
-      </c>
-      <c r="AI6" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ6">
+      <c r="AH6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI6">
         <v>9.375E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:36">
+    <row r="7" spans="1:35">
       <c r="B7">
         <v>4</v>
       </c>
@@ -3660,7 +3639,7 @@
         <v>1.0752025361042621</v>
       </c>
       <c r="K7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.075202536104262E-3</v>
       </c>
       <c r="L7" s="4">
@@ -3683,7 +3662,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S7">
         <v>30</v>
@@ -3693,7 +3672,7 @@
         <v>0.47258333333333336</v>
       </c>
       <c r="U7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>4.6009999999999997E-6</v>
       </c>
       <c r="V7">
@@ -3703,50 +3682,47 @@
       <c r="W7">
         <v>0.43</v>
       </c>
-      <c r="X7" s="4">
-        <f t="shared" si="10"/>
-        <v>0.45838000000000001</v>
+      <c r="X7">
+        <f t="shared" si="6"/>
+        <v>10.32</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="11"/>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z7">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA7">
+        <v>1E-4</v>
+      </c>
+      <c r="AB7" s="21">
+        <v>0</v>
+      </c>
+      <c r="AC7">
+        <v>0</v>
+      </c>
+      <c r="AD7">
+        <v>2E-3</v>
+      </c>
+      <c r="AE7">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AF7">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AG7">
         <v>1</v>
       </c>
-      <c r="AB7">
-        <v>1E-4</v>
-      </c>
-      <c r="AC7" s="21">
-        <v>0</v>
-      </c>
-      <c r="AD7">
-        <v>0</v>
-      </c>
-      <c r="AE7">
-        <v>2E-3</v>
-      </c>
-      <c r="AF7">
-        <v>1E-3</v>
-      </c>
-      <c r="AG7">
-        <f t="shared" si="6"/>
-        <v>1E-3</v>
-      </c>
-      <c r="AH7">
-        <v>1</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ7">
+      <c r="AH7" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI7">
         <v>9.375E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:36">
+    <row r="8" spans="1:35">
       <c r="B8">
         <v>5</v>
       </c>
@@ -3776,14 +3752,14 @@
         <v>1.0752025361042621</v>
       </c>
       <c r="K8">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.075202536104262E-3</v>
       </c>
       <c r="L8" s="4">
         <v>10</v>
       </c>
       <c r="M8">
-        <f t="shared" ref="M8" si="12">L8*J8</f>
+        <f t="shared" ref="M8" si="11">L8*J8</f>
         <v>10.752025361042621</v>
       </c>
       <c r="N8">
@@ -3799,7 +3775,7 @@
         <v>0</v>
       </c>
       <c r="R8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S8">
         <v>30</v>
@@ -3809,7 +3785,7 @@
         <v>0.47258333333333336</v>
       </c>
       <c r="U8">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>4.6009999999999997E-6</v>
       </c>
       <c r="V8">
@@ -3819,50 +3795,47 @@
       <c r="W8">
         <v>0.43</v>
       </c>
-      <c r="X8" s="4">
-        <f t="shared" si="10"/>
-        <v>0.45838000000000001</v>
+      <c r="X8">
+        <f t="shared" si="6"/>
+        <v>10.32</v>
       </c>
       <c r="Y8">
-        <f t="shared" si="11"/>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z8">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA8">
+        <v>1E-4</v>
+      </c>
+      <c r="AB8">
         <v>1</v>
       </c>
-      <c r="AB8">
+      <c r="AC8">
+        <v>0</v>
+      </c>
+      <c r="AD8">
+        <v>2E-3</v>
+      </c>
+      <c r="AE8">
+        <f t="shared" si="7"/>
         <v>1E-4</v>
       </c>
-      <c r="AC8">
+      <c r="AF8">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AG8">
         <v>1</v>
       </c>
-      <c r="AD8">
-        <v>0</v>
-      </c>
-      <c r="AE8">
-        <v>2E-3</v>
-      </c>
-      <c r="AF8">
-        <v>1E-3</v>
-      </c>
-      <c r="AG8">
-        <f t="shared" si="6"/>
-        <v>1E-3</v>
-      </c>
-      <c r="AH8">
-        <v>1</v>
-      </c>
-      <c r="AI8" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ8">
+      <c r="AH8" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI8">
         <v>9.375E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:36">
+    <row r="9" spans="1:35">
       <c r="B9">
         <v>6</v>
       </c>
@@ -3892,7 +3865,7 @@
         <v>1.0752025361042621</v>
       </c>
       <c r="K9">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.075202536104262E-3</v>
       </c>
       <c r="L9" s="4">
@@ -3915,7 +3888,7 @@
         <v>0</v>
       </c>
       <c r="R9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S9">
         <v>30</v>
@@ -3925,7 +3898,7 @@
         <v>0.47258333333333336</v>
       </c>
       <c r="U9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>4.6009999999999997E-6</v>
       </c>
       <c r="V9">
@@ -3935,50 +3908,47 @@
       <c r="W9">
         <v>0.43</v>
       </c>
-      <c r="X9" s="4">
-        <f>W9*1.066</f>
-        <v>0.45838000000000001</v>
+      <c r="X9">
+        <f t="shared" si="6"/>
+        <v>10.32</v>
       </c>
       <c r="Y9">
-        <f>X9 *24</f>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z9">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA9">
+        <v>1E-4</v>
+      </c>
+      <c r="AB9" s="21">
+        <v>0</v>
+      </c>
+      <c r="AC9">
+        <v>0</v>
+      </c>
+      <c r="AD9">
+        <v>2E-3</v>
+      </c>
+      <c r="AE9">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AF9">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AG9">
         <v>1</v>
       </c>
-      <c r="AB9">
-        <v>1E-4</v>
-      </c>
-      <c r="AC9" s="21">
-        <v>0</v>
-      </c>
-      <c r="AD9">
-        <v>0</v>
-      </c>
-      <c r="AE9">
-        <v>2E-3</v>
-      </c>
-      <c r="AF9">
-        <v>1E-3</v>
-      </c>
-      <c r="AG9">
-        <f t="shared" si="6"/>
-        <v>1E-3</v>
-      </c>
-      <c r="AH9">
-        <v>1</v>
-      </c>
-      <c r="AI9" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ9">
+      <c r="AH9" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI9">
         <v>9.375E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:36">
+    <row r="10" spans="1:35">
       <c r="B10">
         <v>7</v>
       </c>
@@ -4004,11 +3974,11 @@
         <v>0.14336033814723495</v>
       </c>
       <c r="J10">
-        <f t="shared" ref="J10:J11" si="13">I10*7.5</f>
+        <f t="shared" ref="J10:J11" si="12">I10*7.5</f>
         <v>1.0752025361042621</v>
       </c>
       <c r="K10">
-        <f t="shared" ref="K10:K11" si="14">J10/1000</f>
+        <f t="shared" ref="K10:K11" si="13">J10/1000</f>
         <v>1.075202536104262E-3</v>
       </c>
       <c r="L10" s="4">
@@ -4031,7 +4001,7 @@
         <v>0</v>
       </c>
       <c r="R10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S10">
         <v>30</v>
@@ -4040,7 +4010,7 @@
         <v>1E-3</v>
       </c>
       <c r="U10">
-        <f t="shared" ref="U10:U13" si="15">4.3 /1000000 *1.07</f>
+        <f t="shared" ref="U10:U13" si="14">4.3 /1000000 *1.07</f>
         <v>4.6009999999999997E-6</v>
       </c>
       <c r="V10">
@@ -4050,50 +4020,47 @@
       <c r="W10">
         <v>0.43</v>
       </c>
-      <c r="X10" s="4">
-        <f>W10*1.066</f>
-        <v>0.45838000000000001</v>
+      <c r="X10">
+        <f t="shared" si="6"/>
+        <v>10.32</v>
       </c>
       <c r="Y10">
-        <f>X10 *24</f>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z10">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA10">
+        <v>1E-4</v>
+      </c>
+      <c r="AB10">
         <v>1</v>
       </c>
-      <c r="AB10">
+      <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>2E-3</v>
+      </c>
+      <c r="AE10">
+        <f t="shared" si="7"/>
         <v>1E-4</v>
       </c>
-      <c r="AC10">
+      <c r="AF10">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AG10">
         <v>1</v>
       </c>
-      <c r="AD10">
-        <v>0</v>
-      </c>
-      <c r="AE10">
-        <v>2E-3</v>
-      </c>
-      <c r="AF10">
-        <v>1E-3</v>
-      </c>
-      <c r="AG10">
-        <f t="shared" si="6"/>
-        <v>1E-3</v>
-      </c>
-      <c r="AH10">
-        <v>1</v>
-      </c>
-      <c r="AI10" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ10">
+      <c r="AH10" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI10">
         <v>9.375E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:36">
+    <row r="11" spans="1:35">
       <c r="B11">
         <v>8</v>
       </c>
@@ -4119,11 +4086,11 @@
         <v>0.14336033814723495</v>
       </c>
       <c r="J11">
+        <f t="shared" si="12"/>
+        <v>1.0752025361042621</v>
+      </c>
+      <c r="K11">
         <f t="shared" si="13"/>
-        <v>1.0752025361042621</v>
-      </c>
-      <c r="K11">
-        <f t="shared" si="14"/>
         <v>1.075202536104262E-3</v>
       </c>
       <c r="L11" s="4">
@@ -4146,7 +4113,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S11">
         <v>30</v>
@@ -4155,7 +4122,7 @@
         <v>0.8</v>
       </c>
       <c r="U11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>4.6009999999999997E-6</v>
       </c>
       <c r="V11">
@@ -4165,50 +4132,47 @@
       <c r="W11">
         <v>0.43</v>
       </c>
-      <c r="X11" s="4">
-        <f>W11*1.066</f>
-        <v>0.45838000000000001</v>
+      <c r="X11">
+        <f t="shared" si="6"/>
+        <v>10.32</v>
       </c>
       <c r="Y11">
-        <f>X11 *24</f>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z11">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA11">
+        <v>1E-4</v>
+      </c>
+      <c r="AB11">
         <v>1</v>
       </c>
-      <c r="AB11">
+      <c r="AC11">
+        <v>0</v>
+      </c>
+      <c r="AD11">
+        <v>2E-3</v>
+      </c>
+      <c r="AE11">
+        <f t="shared" si="7"/>
         <v>1E-4</v>
       </c>
-      <c r="AC11">
+      <c r="AF11">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AG11">
         <v>1</v>
       </c>
-      <c r="AD11">
-        <v>0</v>
-      </c>
-      <c r="AE11">
-        <v>2E-3</v>
-      </c>
-      <c r="AF11">
-        <v>1E-3</v>
-      </c>
-      <c r="AG11">
-        <f t="shared" si="6"/>
-        <v>1E-3</v>
-      </c>
-      <c r="AH11">
-        <v>1</v>
-      </c>
-      <c r="AI11" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ11">
+      <c r="AH11" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI11">
         <v>9.375E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:36">
+    <row r="12" spans="1:35">
       <c r="B12">
         <v>9</v>
       </c>
@@ -4234,11 +4198,11 @@
         <v>0.14336033814723495</v>
       </c>
       <c r="J12">
-        <f t="shared" ref="J12:J13" si="16">I12*7.5</f>
+        <f t="shared" ref="J12:J13" si="15">I12*7.5</f>
         <v>1.0752025361042621</v>
       </c>
       <c r="K12">
-        <f t="shared" ref="K12:K13" si="17">J12/1000</f>
+        <f t="shared" ref="K12:K13" si="16">J12/1000</f>
         <v>1.075202536104262E-3</v>
       </c>
       <c r="L12" s="4">
@@ -4261,17 +4225,17 @@
         <v>0</v>
       </c>
       <c r="R12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S12">
         <v>30</v>
       </c>
       <c r="T12">
-        <f t="shared" ref="T12:T13" si="18">10.6/12*1.07/2</f>
+        <f t="shared" ref="T12:T13" si="17">10.6/12*1.07/2</f>
         <v>0.47258333333333336</v>
       </c>
       <c r="U12">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>4.6009999999999997E-6</v>
       </c>
       <c r="V12">
@@ -4281,50 +4245,47 @@
       <c r="W12">
         <v>0.43</v>
       </c>
-      <c r="X12" s="4">
-        <f>W12*1.066</f>
-        <v>0.45838000000000001</v>
+      <c r="X12">
+        <f t="shared" si="6"/>
+        <v>10.32</v>
       </c>
       <c r="Y12">
-        <f>X12 *24</f>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z12">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA12">
+        <v>1E-4</v>
+      </c>
+      <c r="AB12">
         <v>1</v>
       </c>
-      <c r="AB12">
+      <c r="AC12">
+        <v>0</v>
+      </c>
+      <c r="AD12">
+        <v>2E-3</v>
+      </c>
+      <c r="AE12">
+        <f t="shared" si="7"/>
         <v>1E-4</v>
       </c>
-      <c r="AC12">
+      <c r="AF12">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AG12">
         <v>1</v>
       </c>
-      <c r="AD12">
-        <v>0</v>
-      </c>
-      <c r="AE12">
-        <v>2E-3</v>
-      </c>
-      <c r="AF12">
-        <v>1E-3</v>
-      </c>
-      <c r="AG12">
-        <f t="shared" si="6"/>
-        <v>1E-3</v>
-      </c>
-      <c r="AH12">
-        <v>1</v>
-      </c>
-      <c r="AI12" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ12">
+      <c r="AH12" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI12">
         <v>9.375E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:36">
+    <row r="13" spans="1:35">
       <c r="B13">
         <v>10</v>
       </c>
@@ -4350,11 +4311,11 @@
         <v>0.14336033814723495</v>
       </c>
       <c r="J13">
+        <f t="shared" si="15"/>
+        <v>1.0752025361042621</v>
+      </c>
+      <c r="K13">
         <f t="shared" si="16"/>
-        <v>1.0752025361042621</v>
-      </c>
-      <c r="K13">
-        <f t="shared" si="17"/>
         <v>1.075202536104262E-3</v>
       </c>
       <c r="L13" s="4">
@@ -4377,17 +4338,17 @@
         <v>0</v>
       </c>
       <c r="R13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="S13">
         <v>30</v>
       </c>
       <c r="T13">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>0.47258333333333336</v>
       </c>
       <c r="U13">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>4.6009999999999997E-6</v>
       </c>
       <c r="V13">
@@ -4397,51 +4358,48 @@
       <c r="W13">
         <v>0.43</v>
       </c>
-      <c r="X13" s="4">
-        <f>W13*1.066</f>
-        <v>0.45838000000000001</v>
+      <c r="X13">
+        <f t="shared" si="6"/>
+        <v>10.32</v>
       </c>
       <c r="Y13">
-        <f>X13 *24</f>
-        <v>11.00112</v>
+        <v>0.06</v>
       </c>
       <c r="Z13">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="AA13">
+        <v>1E-4</v>
+      </c>
+      <c r="AB13">
         <v>1</v>
       </c>
-      <c r="AB13">
+      <c r="AC13">
+        <v>0</v>
+      </c>
+      <c r="AD13">
+        <v>2E-3</v>
+      </c>
+      <c r="AE13">
+        <f t="shared" si="7"/>
         <v>1E-4</v>
       </c>
-      <c r="AC13">
+      <c r="AF13">
+        <f t="shared" si="7"/>
+        <v>1E-4</v>
+      </c>
+      <c r="AG13">
         <v>1</v>
       </c>
-      <c r="AD13">
-        <v>0</v>
-      </c>
-      <c r="AE13">
-        <v>2E-3</v>
-      </c>
-      <c r="AF13">
-        <v>1E-3</v>
-      </c>
-      <c r="AG13">
-        <f t="shared" si="6"/>
-        <v>1E-3</v>
-      </c>
-      <c r="AH13">
-        <v>1</v>
-      </c>
-      <c r="AI13" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ13">
+      <c r="AH13" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI13">
         <v>9.375E-2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:AJ3" xr:uid="{AB7B919E-F4BE-8A4F-9679-A3F32BFB830E}"/>
+  <autoFilter ref="A3:AI3" xr:uid="{AB7B919E-F4BE-8A4F-9679-A3F32BFB830E}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -4459,7 +4417,7 @@
   <sheetData>
     <row r="1" spans="2:21">
       <c r="B1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="2:21">
@@ -4542,38 +4500,38 @@
     </row>
     <row r="16" spans="2:21">
       <c r="L16" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="12:20">
       <c r="L17" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N17" t="s">
+        <v>32</v>
+      </c>
+      <c r="O17" t="s">
+        <v>36</v>
+      </c>
+      <c r="P17" t="s">
         <v>33</v>
       </c>
-      <c r="O17" t="s">
-        <v>37</v>
-      </c>
-      <c r="P17" t="s">
+      <c r="Q17" t="s">
         <v>34</v>
       </c>
-      <c r="Q17" t="s">
+      <c r="R17" t="s">
         <v>35</v>
       </c>
-      <c r="R17" t="s">
-        <v>36</v>
-      </c>
       <c r="T17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="12:20">
       <c r="L18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="N18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O18">
         <v>9</v>
@@ -4594,12 +4552,12 @@
     </row>
     <row r="19" spans="12:20">
       <c r="L19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="12:20">
       <c r="L20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="12:20">
@@ -4608,43 +4566,43 @@
         <v>227</v>
       </c>
       <c r="M21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="12:20">
       <c r="L22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="12:20">
       <c r="L25" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N25" t="s">
+        <v>32</v>
+      </c>
+      <c r="O25" t="s">
+        <v>36</v>
+      </c>
+      <c r="P25" t="s">
         <v>33</v>
       </c>
-      <c r="O25" t="s">
-        <v>37</v>
-      </c>
-      <c r="P25" t="s">
+      <c r="Q25" t="s">
         <v>34</v>
       </c>
-      <c r="Q25" t="s">
+      <c r="R25" t="s">
         <v>35</v>
       </c>
-      <c r="R25" t="s">
-        <v>36</v>
-      </c>
       <c r="T25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="12:20">
       <c r="L26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O26">
         <v>2</v>
@@ -4668,53 +4626,53 @@
         <v>60</v>
       </c>
       <c r="M27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="12:20">
       <c r="L28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" spans="12:20">
       <c r="L31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="32" spans="12:20" ht="18">
       <c r="L32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="10:20">
       <c r="L33" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N33" t="s">
+        <v>32</v>
+      </c>
+      <c r="O33" t="s">
+        <v>36</v>
+      </c>
+      <c r="P33" t="s">
         <v>33</v>
       </c>
-      <c r="O33" t="s">
-        <v>37</v>
-      </c>
-      <c r="P33" t="s">
+      <c r="Q33" t="s">
         <v>34</v>
       </c>
-      <c r="Q33" t="s">
+      <c r="R33" t="s">
         <v>35</v>
       </c>
-      <c r="R33" t="s">
-        <v>36</v>
-      </c>
       <c r="T33" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" spans="10:20">
       <c r="L34" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N34" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O34">
         <v>1</v>
@@ -4737,7 +4695,7 @@
       <c r="J35" s="11"/>
       <c r="K35" s="10"/>
       <c r="L35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="10:20">
@@ -4755,7 +4713,7 @@
     </row>
     <row r="40" spans="10:20">
       <c r="M40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41" spans="10:20">
@@ -4763,25 +4721,25 @@
         <v>2.6</v>
       </c>
       <c r="N41" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P41">
         <v>2.6</v>
       </c>
       <c r="Q41" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="42" spans="10:20">
       <c r="L42" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M42">
         <f>12+1.8+0.5*16+0.2*14</f>
         <v>24.6</v>
       </c>
       <c r="N42" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="48" spans="10:20">
@@ -4792,7 +4750,7 @@
         <v>1</v>
       </c>
       <c r="N50" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="51" spans="3:14">
@@ -4801,10 +4759,10 @@
         <v>0.14336033814723495</v>
       </c>
       <c r="M51" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N51" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="54" spans="3:14">
@@ -4813,7 +4771,7 @@
         <v>2.032520325203252E-10</v>
       </c>
       <c r="M54" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" spans="3:14">
@@ -4830,81 +4788,81 @@
     </row>
     <row r="58" spans="3:14">
       <c r="L58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="59" spans="3:14" ht="18">
       <c r="L59" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="60" spans="3:14">
       <c r="C60" t="s">
+        <v>89</v>
+      </c>
+      <c r="D60" t="s">
         <v>90</v>
       </c>
-      <c r="D60" t="s">
-        <v>91</v>
-      </c>
       <c r="L60" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M60">
         <f>5*12+7+2*16+14</f>
         <v>113</v>
       </c>
       <c r="N60" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="61" spans="3:14">
       <c r="D61" t="s">
+        <v>91</v>
+      </c>
+      <c r="E61" t="s">
         <v>92</v>
       </c>
-      <c r="E61" t="s">
-        <v>93</v>
-      </c>
       <c r="L61" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="62" spans="3:14">
       <c r="C62" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D62">
         <v>7.5</v>
       </c>
       <c r="E62" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L62" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="63" spans="3:14">
       <c r="C63" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D63">
         <v>5.9</v>
       </c>
       <c r="E63" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L63" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="64" spans="3:14">
       <c r="C64" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D64" s="13">
         <f>D62-D63</f>
         <v>1.5999999999999996</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F64" s="13"/>
       <c r="K64">
@@ -4912,117 +4870,117 @@
         <v>4.25</v>
       </c>
       <c r="L64" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="65" spans="3:13">
       <c r="C65" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D65" s="13">
         <f>D62+D63</f>
         <v>13.4</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F65" s="13"/>
       <c r="L65" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="66" spans="3:13">
       <c r="C66" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D66">
         <f>D62/227.172/1000</f>
         <v>3.3014632084940045E-5</v>
       </c>
       <c r="E66" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L66">
         <f>4.25*32</f>
         <v>136</v>
       </c>
       <c r="M66" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="67" spans="3:13">
       <c r="C67" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D67">
         <f>D63/227.172/1000</f>
         <v>2.5971510573486172E-5</v>
       </c>
       <c r="E67" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L67">
         <f>L66/M60</f>
         <v>1.2035398230088497</v>
       </c>
       <c r="M67" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="68" spans="3:13">
       <c r="C68" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D68">
         <f>D66*24.6</f>
         <v>8.1215994928952515E-4</v>
       </c>
       <c r="E68" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L68" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="69" spans="3:13">
       <c r="C69" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D69">
         <f>D67*24.6</f>
         <v>6.388991601077599E-4</v>
       </c>
       <c r="E69" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70" spans="3:13">
       <c r="C70" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D70">
         <f>D68*1.075/1.05</f>
         <v>8.3149709093927569E-4</v>
       </c>
       <c r="E70" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="71" spans="3:13">
       <c r="C71" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D71">
         <f>D69*1.075/1.05</f>
         <v>6.5411104487223025E-4</v>
       </c>
       <c r="E71" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="75" spans="3:13">
       <c r="C75" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="76" spans="3:13">
@@ -5030,7 +4988,7 @@
         <v>0.33</v>
       </c>
       <c r="E76" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="77" spans="3:13">
@@ -5038,7 +4996,7 @@
         <v>0.73</v>
       </c>
       <c r="E77" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="78" spans="3:13">
@@ -5047,7 +5005,7 @@
         <v>3.3000000000000002E-7</v>
       </c>
       <c r="E78" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="79" spans="3:13">
@@ -5056,7 +5014,7 @@
         <v>7.3E-7</v>
       </c>
       <c r="E79" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="80" spans="3:13">
@@ -5065,7 +5023,7 @@
         <v>2.7500000000000001E-8</v>
       </c>
       <c r="E80" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="81" spans="4:12">
@@ -5074,7 +5032,7 @@
         <v>6.0833333333333329E-8</v>
       </c>
       <c r="E81" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="82" spans="4:12">
@@ -5083,7 +5041,7 @@
         <v>5.5000000000000014E-3</v>
       </c>
       <c r="E82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="83" spans="4:12">
@@ -5092,7 +5050,7 @@
         <v>1.2166666666666666E-2</v>
       </c>
       <c r="E83" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="84" spans="4:12">
@@ -5101,7 +5059,7 @@
         <v>0.13530000000000003</v>
       </c>
       <c r="E84" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="85" spans="4:12">
@@ -5110,7 +5068,7 @@
         <v>0.29930000000000001</v>
       </c>
       <c r="E85" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="86" spans="4:12">
@@ -5119,7 +5077,7 @@
         <v>0.12885714285714289</v>
       </c>
       <c r="E86" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="87" spans="4:12">
@@ -5128,7 +5086,7 @@
         <v>0.28504761904761905</v>
       </c>
       <c r="E87" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="89" spans="4:12">
@@ -5137,10 +5095,10 @@
         <v>8.4242681454371637E-2</v>
       </c>
       <c r="E89" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K89" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="90" spans="4:12">
@@ -5148,13 +5106,13 @@
         <v>6.905E-6</v>
       </c>
       <c r="E90" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K90">
         <v>0.35</v>
       </c>
       <c r="L90" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="91" spans="4:12">
@@ -5163,14 +5121,14 @@
         <v>5.8169571544243611E-7</v>
       </c>
       <c r="E91" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K91">
         <f>K90/1000000/24.6</f>
         <v>1.4227642276422762E-8</v>
       </c>
       <c r="L91" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="92" spans="4:12">
@@ -5179,14 +5137,14 @@
         <v>5.8169571544243611E-7</v>
       </c>
       <c r="E92" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="K92">
         <f>K91*1.05</f>
         <v>1.4939024390243901E-8</v>
       </c>
       <c r="L92" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="93" spans="4:12">
@@ -5195,7 +5153,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="L93" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="94" spans="4:12">
@@ -5204,12 +5162,12 @@
         <v>1.4939024390243901E-3</v>
       </c>
       <c r="L94" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="96" spans="4:12">
       <c r="E96" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="97" spans="4:14">
@@ -5217,7 +5175,7 @@
         <v>0.33500000000000002</v>
       </c>
       <c r="E97" s="17" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="98" spans="4:14">
@@ -5225,13 +5183,13 @@
         <v>9.09</v>
       </c>
       <c r="E98" t="s">
+        <v>120</v>
+      </c>
+      <c r="F98" t="s">
         <v>121</v>
       </c>
-      <c r="F98" t="s">
-        <v>122</v>
-      </c>
       <c r="L98" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="99" spans="4:14">
@@ -5239,20 +5197,20 @@
         <v>7.58</v>
       </c>
       <c r="E99" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F99" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L99">
         <f>AVERAGE(D127, D86:D87,D70)</f>
         <v>0.10371468607138892</v>
       </c>
       <c r="M99" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N99" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="100" spans="4:14">
@@ -5260,13 +5218,13 @@
         <v>7.96</v>
       </c>
       <c r="E100" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F100" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="N100" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="101" spans="4:14">
@@ -5274,10 +5232,10 @@
         <v>6.52</v>
       </c>
       <c r="E101" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F101" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="102" spans="4:14">
@@ -5285,10 +5243,10 @@
         <v>4.71</v>
       </c>
       <c r="E102" s="17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F102" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H102">
         <f>AVERAGE(D102:D105)</f>
@@ -5300,10 +5258,10 @@
         <v>4.3499999999999996</v>
       </c>
       <c r="E103" s="17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F103" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="104" spans="4:14">
@@ -5311,10 +5269,10 @@
         <v>4.18</v>
       </c>
       <c r="E104" s="17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F104" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="105" spans="4:14">
@@ -5322,10 +5280,10 @@
         <v>4.13</v>
       </c>
       <c r="E105" s="17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F105" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="106" spans="4:14">
@@ -5333,7 +5291,7 @@
         <v>4.3</v>
       </c>
       <c r="E106" s="17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="107" spans="4:14">
@@ -5341,7 +5299,7 @@
         <v>0.5</v>
       </c>
       <c r="E107" s="17" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="108" spans="4:14">
@@ -5349,7 +5307,7 @@
         <v>14.9</v>
       </c>
       <c r="E108" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="109" spans="4:14">
@@ -5357,7 +5315,7 @@
         <v>1.9</v>
       </c>
       <c r="E109" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="110" spans="4:14">
@@ -5365,7 +5323,7 @@
         <v>12.4</v>
       </c>
       <c r="E110" s="17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="111" spans="4:14">
@@ -5373,7 +5331,7 @@
         <v>1.2</v>
       </c>
       <c r="E111" s="17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="112" spans="4:14">
@@ -5381,7 +5339,7 @@
         <v>0.01</v>
       </c>
       <c r="E112" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="113" spans="4:5">
@@ -5389,7 +5347,7 @@
         <v>8.1</v>
       </c>
       <c r="E113" s="17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="114" spans="4:5">
@@ -5397,12 +5355,12 @@
         <v>0.15336312500000002</v>
       </c>
       <c r="E114" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="115" spans="4:5">
       <c r="E115" s="17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="116" spans="4:5">
@@ -5411,7 +5369,7 @@
         <v>8.3333333333333344E-7</v>
       </c>
       <c r="E116" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="117" spans="4:5">
@@ -5420,7 +5378,7 @@
         <v>6.7499999999999993E-4</v>
       </c>
       <c r="E117" s="17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="118" spans="4:5">
@@ -5429,7 +5387,7 @@
         <v>1.2780260416666668E-5</v>
       </c>
       <c r="E118" s="17" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="119" spans="4:5">
@@ -5438,7 +5396,7 @@
         <v>1.9190174630589144E-7</v>
       </c>
       <c r="E119" s="17" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="120" spans="4:5">
@@ -5447,7 +5405,7 @@
         <v>1.5544041450777204E-4</v>
       </c>
       <c r="E120" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="121" spans="4:5">
@@ -5456,7 +5414,7 @@
         <v>2.9430651506428716E-6</v>
       </c>
       <c r="E121" s="17" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="122" spans="4:5">
@@ -5465,7 +5423,7 @@
         <v>7.8008839961744482E-6</v>
       </c>
       <c r="E122" s="17" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="123" spans="4:5">
@@ -5474,7 +5432,7 @@
         <v>6.3187160369013026E-3</v>
       </c>
       <c r="E123" s="17" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="124" spans="4:5">
@@ -5483,7 +5441,7 @@
         <v>1.1963679474158013E-4</v>
       </c>
       <c r="E124" s="17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="125" spans="4:5">
@@ -5492,7 +5450,7 @@
         <v>7.9866193294166962E-6</v>
       </c>
       <c r="E125" s="17" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="126" spans="4:5">
@@ -5501,7 +5459,7 @@
         <v>6.4691616568275231E-3</v>
       </c>
       <c r="E126" s="17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="127" spans="4:5">
@@ -5510,12 +5468,12 @@
         <v>1.224852898544749E-4</v>
       </c>
       <c r="E127" s="17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="130" spans="4:6" ht="198">
       <c r="D130" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="131" spans="4:6">
@@ -5524,10 +5482,10 @@
         <v>1.6000000000000003E-5</v>
       </c>
       <c r="E131" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F131" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="132" spans="4:6">
@@ -5536,10 +5494,10 @@
         <v>4.5714285714285719E-6</v>
       </c>
       <c r="E132" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F132" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="133" spans="4:6">
@@ -5547,10 +5505,10 @@
         <v>630000</v>
       </c>
       <c r="E133" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F133" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="134" spans="4:6">
@@ -5559,10 +5517,10 @@
         <v>6.3E+17</v>
       </c>
       <c r="E134" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F134" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="135" spans="4:6">
@@ -5571,10 +5529,10 @@
         <v>2880000000000.0005</v>
       </c>
       <c r="E135" t="s">
+        <v>165</v>
+      </c>
+      <c r="F135" t="s">
         <v>166</v>
-      </c>
-      <c r="F135" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="136" spans="4:6">
@@ -5583,10 +5541,10 @@
         <v>227</v>
       </c>
       <c r="E136" t="s">
+        <v>168</v>
+      </c>
+      <c r="F136" t="s">
         <v>169</v>
-      </c>
-      <c r="F136" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="137" spans="4:6">
@@ -5595,10 +5553,10 @@
         <v>653760000000000.13</v>
       </c>
       <c r="E137" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F137" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="138" spans="4:6">
@@ -5607,10 +5565,10 @@
         <v>653760000000.00012</v>
       </c>
       <c r="E138" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F138" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="139" spans="4:6">
@@ -5619,10 +5577,10 @@
         <v>653760000.00000012</v>
       </c>
       <c r="E139" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F139" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>